<commit_message>
R2.9: SCALE base vuelve a 981 y .STD escalado
El .STD R2.9 usa la lista de diseno ya dividida entre R (meseta 0.2057 g)
con SCALE 981, asi que COEFICIENTE C77:D77 vuelve a ser la captura 981.
SCALE nuevo = 981 x factor: 1623.729 en X (casos 4 y 6) y 1131.192 en Z
(casos 5 y 7), aplicado en 001_NOSE_DOCK_H5_H6_R2.9_ESCALADO.STD.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DXC88k2xtfXzDpyA8FhCSg
</commit_message>
<xml_diff>
--- a/EspectrosSismo_Naves_ElSalvador_NTDS_ASCE_STAAD_R2.9_REVISADO.xlsx
+++ b/EspectrosSismo_Naves_ElSalvador_NTDS_ASCE_STAAD_R2.9_REVISADO.xlsx
@@ -14066,7 +14066,7 @@
       </c>
       <c r="F76" s="52" t="inlineStr">
         <is>
-          <t>◀ ESTE ES EL FACTOR QUE MULTIPLICA TU ESPECTRO (X en los casos 4 y 6; Z en los casos 5 y 7). Se aplica al SCALE que ya tienes en el .STD, no al 981. 1.000 si ya pasa. Sube en la misma proporción todo lo del sismo: fuerzas, momentos, reacciones y desplazamientos.</t>
+          <t>◀ ESTE ES EL FACTOR. Multiplica el SCALE que ya tienes en el .STD (981 en el R2.9): SCALE nuevo = 981 × factor (fila 78). No es meter otra vez 981 encima: el 981 sólo pasa de g a cm/s². X en los casos 4 y 6; Z en los casos 5 y 7. Sube en la misma proporción todo lo del sismo: fuerzas, momentos, reacciones y desplazamientos.</t>
         </is>
       </c>
       <c r="G76" s="48" t="inlineStr">
@@ -14081,13 +14081,11 @@
           <t>SCALE que traes en el .STD</t>
         </is>
       </c>
-      <c r="C77" s="13">
-        <f>STAAD!$C$18</f>
-        <v>140.095</v>
-      </c>
-      <c r="D77" s="13">
-        <f>STAAD!$D$18</f>
-        <v>140.095</v>
+      <c r="C77" s="16">
+        <v>981</v>
+      </c>
+      <c r="D77" s="16">
+        <v>981</v>
       </c>
       <c r="E77" s="6" t="inlineStr">
         <is>
@@ -14096,12 +14094,12 @@
       </c>
       <c r="F77" s="44" t="inlineStr">
         <is>
-          <t>CALCULADA (antes era una captura fija de 981 y estaba mal para tu .STD). Es el SCALE de la hoja STAAD (C18) y el que tiene tu .STD: 980.665 / R = 980.665 / 7 = 140.095, porque la lista que pegaste es la ELÁSTICA (meseta 1.44 g). El 981 ya va adentro: no lo vuelvas a meter. Sólo si pegaras la lista de DISEÑO (÷R, meseta 0.2057 g) el SCALE sería 981.</t>
+          <t>CAPTURA. El SCALE que hoy tienen los SPECTRUM de tu .STD. R2.9: 981, porque la lista que pegaste ya viene en g y dividida entre R (meseta 0.2057 g); el 981 sólo convierte g a cm/s². Si usas la lista ELÁSTICA de la hoja STAAD (meseta 1.44 g, como el R3.2), aquí va 140.095 = 980.665/7.</t>
         </is>
       </c>
       <c r="G77" s="48" t="inlineStr">
         <is>
-          <t>Archivo .STD · hoja STAAD, C18</t>
+          <t>Archivo .STD (R2.9: líneas 565, 585, 605 y 625)</t>
         </is>
       </c>
     </row>
@@ -14113,11 +14111,11 @@
       </c>
       <c r="C78" s="21">
         <f>$C$77*$C$76</f>
-        <v>231.8821412634519</v>
+        <v>1623.7294734247916</v>
       </c>
       <c r="D78" s="21">
         <f>$D$77*$D$76</f>
-        <v>161.54371831594693</v>
+        <v>1131.1923171272592</v>
       </c>
       <c r="E78" s="6" t="inlineStr">
         <is>
@@ -14126,7 +14124,7 @@
       </c>
       <c r="F78" s="44" t="inlineStr">
         <is>
-          <t>CALCULADA = 140.095 × factor. Es el número que escribes en SPECTRUM ... ACC SCALE: X en los casos 4 y 6; Z en los casos 5 y 7.</t>
+          <t>CALCULADA = SCALE actual × factor. Es el número que escribes en SPECTRUM ... ACC SCALE: X en los casos 4 y 6; Z en los casos 5 y 7.</t>
         </is>
       </c>
       <c r="G78" s="48" t="inlineStr">
@@ -14750,7 +14748,7 @@
     <row r="103" ht="30" customHeight="1">
       <c r="B103" s="45" t="inlineStr">
         <is>
-          <t>Las dos formas de meterlo en STAAD dan lo mismo</t>
+          <t>Cómo meter el factor en STAAD (las dos formas dan lo mismo)</t>
         </is>
       </c>
       <c r="C103" s="45" t="inlineStr">
@@ -14782,16 +14780,16 @@
     <row r="104" ht="42" customHeight="1">
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>Con TU lista elástica (meseta 1.44 g): SCALE nuevo</t>
+          <t>R2.9 — lista de DISEÑO ÷R (meseta 0.2057 g), SCALE 981: SCALE nuevo</t>
         </is>
       </c>
       <c r="C104" s="13">
         <f>$C$78</f>
-        <v>231.8821412634519</v>
+        <v>1623.7294734247916</v>
       </c>
       <c r="D104" s="13">
         <f>$D$78</f>
-        <v>161.54371831594693</v>
+        <v>1131.1923171272592</v>
       </c>
       <c r="E104" s="6" t="inlineStr">
         <is>
@@ -14800,7 +14798,7 @@
       </c>
       <c r="F104" s="44" t="inlineStr">
         <is>
-          <t>140.095 × factor. Es lo que va en tu .STD.</t>
+          <t>981 × factor. Es lo que va en tu .STD R2.9.</t>
         </is>
       </c>
       <c r="G104" s="48" t="inlineStr">
@@ -14812,16 +14810,16 @@
     <row r="105" ht="42" customHeight="1">
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t>Con la lista de DISEÑO ÷R (meseta 0.2057 g): SCALE</t>
+          <t>Lista ELÁSTICA de la hoja STAAD (meseta 1.44 g), SCALE 140.095: SCALE nuevo</t>
         </is>
       </c>
       <c r="C105" s="13">
-        <f>980.665*$C$76</f>
-        <v>1623.1749888441634</v>
+        <f>STAAD!$C$18*$C$76</f>
+        <v>231.88214126345176</v>
       </c>
       <c r="D105" s="13">
-        <f>980.665*$D$76</f>
-        <v>1130.8060282116285</v>
+        <f>STAAD!$D$18*$D$76</f>
+        <v>161.54371831594636</v>
       </c>
       <c r="E105" s="6" t="inlineStr">
         <is>
@@ -14830,12 +14828,12 @@
       </c>
       <c r="F105" s="44" t="inlineStr">
         <is>
-          <t>981 × factor. Sólo si pegas la lista ya dividida entre R (como la columna J de él). NO lo uses con tu lista elástica: saldría 7 veces más grande.</t>
+          <t>140.095 × factor. Sólo si pegas la lista elástica (como el R3.2). NO lo mezcles con la lista ÷R del R2.9: saldría 7 veces más chico.</t>
         </is>
       </c>
       <c r="G105" s="48" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Hoja STAAD, C18</t>
         </is>
       </c>
     </row>
@@ -14846,12 +14844,12 @@
         </is>
       </c>
       <c r="C106" s="55">
-        <f>DATOS!$C$26*$C$78/980.665</f>
-        <v>0.34049372968278746</v>
+        <f>DATOS!$C$26/$C$12*$C$76</f>
+        <v>0.34049372968278724</v>
       </c>
       <c r="D106" s="55">
-        <f>DATOS!$C$26*$D$78/980.665</f>
-        <v>0.23720939808697525</v>
+        <f>DATOS!$C$26/$D$12*$D$76</f>
+        <v>0.23720939808697442</v>
       </c>
       <c r="E106" s="6" t="inlineStr">
         <is>
@@ -14860,7 +14858,7 @@
       </c>
       <c r="F106" s="44" t="inlineStr">
         <is>
-          <t>= 0.2057 × factor. Las dos formas de arriba dan este mismo valor.</t>
+          <t>= 0.2057 g × factor. Las dos formas de arriba dan esta misma meseta.</t>
         </is>
       </c>
       <c r="G106" s="48" t="inlineStr">

</xml_diff>

<commit_message>
R2.9: W sismico 17.13 t (peso de STAAD); factor X 1.621, Z 1.129
SCALE nuevo 1590.308 (X, casos 4 y 6) y 1107.909 (Z, casos 5 y 7).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DXC88k2xtfXzDpyA8FhCSg
</commit_message>
<xml_diff>
--- a/EspectrosSismo_Naves_ElSalvador_NTDS_ASCE_STAAD_R2.9_REVISADO.xlsx
+++ b/EspectrosSismo_Naves_ElSalvador_NTDS_ASCE_STAAD_R2.9_REVISADO.xlsx
@@ -12433,13 +12433,15 @@
         <v>167</v>
       </c>
       <c r="C60" s="15">
-        <v>17.489999999999998</v>
+        <v>17.13</v>
       </c>
       <c r="D60" s="6" t="s">
         <v>168</v>
       </c>
-      <c r="E60" s="3" t="s">
-        <v>876</v>
+      <c r="E60" s="3" t="inlineStr">
+        <is>
+          <t>CAPTURA. 17.13 t = peso sísmico que reporta STAAD (el mismo que usa ANALISIS_CARGAS_NAVE, 17,129 kg), para que el V mínimo y el V modal salgan de la misma masa. Antes: 17.49 t por áreas tributarias (acero 11.82 + CM techo 3.12 + CM muros 2.15 + cortina 0.40).</t>
+        </is>
       </c>
       <c r="F60" s="4" t="s">
         <v>169</v>
@@ -12450,13 +12452,15 @@
         <v>170</v>
       </c>
       <c r="C61" s="15">
-        <v>17.489999999999998</v>
+        <v>17.13</v>
       </c>
       <c r="D61" s="6" t="s">
         <v>168</v>
       </c>
-      <c r="E61" s="3" t="s">
-        <v>877</v>
+      <c r="E61" s="3" t="inlineStr">
+        <is>
+          <t>CAPTURA. Igual que la NTDS: 17.13 t (fuera del AMSS sólo es referencia).</t>
+        </is>
       </c>
       <c r="F61" s="4" t="s">
         <v>171</v>
@@ -13010,11 +13014,11 @@
       </c>
       <c r="C24" s="21">
         <f>$C$23*DATOS!$C$60</f>
-        <v>2.91444057808651</v>
+        <v>2.8544520927742667</v>
       </c>
       <c r="D24" s="21">
         <f>$D$23*DATOS!$C$60</f>
-        <v>3.49389675932274</v>
+        <v>3.421981217106834</v>
       </c>
       <c r="E24" s="6" t="s">
         <v>168</v>
@@ -13557,11 +13561,11 @@
       </c>
       <c r="C51" s="21">
         <f>$C$50*DATOS!$C$61</f>
-        <v>8.54045028571428</v>
+        <v>8.36466057142857</v>
       </c>
       <c r="D51" s="21">
         <f>$D$50*DATOS!$C$61</f>
-        <v>8.54045028571428</v>
+        <v>8.36466057142857</v>
       </c>
       <c r="E51" s="6" t="s">
         <v>168</v>
@@ -13708,11 +13712,11 @@
       </c>
       <c r="C60" s="13">
         <f>$C$24*DATOS!$C$12</f>
-        <v>4.16765002666371</v>
+        <v>4.081866492667201</v>
       </c>
       <c r="D60" s="13">
         <f>$D$24*DATOS!$C$12</f>
-        <v>4.99627236583152</v>
+        <v>4.893433140462772</v>
       </c>
       <c r="E60" s="6" t="s">
         <v>168</v>
@@ -13730,11 +13734,11 @@
       </c>
       <c r="C61" s="13">
         <f>$C$51</f>
-        <v>8.54045028571428</v>
+        <v>8.36466057142857</v>
       </c>
       <c r="D61" s="13">
         <f>$D$51</f>
-        <v>8.54045028571428</v>
+        <v>8.36466057142857</v>
       </c>
       <c r="E61" s="6" t="s">
         <v>168</v>
@@ -13993,11 +13997,11 @@
       </c>
       <c r="C74" s="13">
         <f>$C$27*DATOS!$C$60</f>
-        <v>2.87835428571429</v>
+        <v>2.8191085714285715</v>
       </c>
       <c r="D74" s="13">
         <f>$D$27*DATOS!$C$60</f>
-        <v>3.14450708339047</v>
+        <v>3.0797830953961505</v>
       </c>
       <c r="E74" s="6" t="inlineStr">
         <is>
@@ -14053,11 +14057,11 @@
       </c>
       <c r="C76" s="50">
         <f>IF($C$73&gt;0,MAX(1,$C$74/$C$73),1)</f>
-        <v>1.65517785262466</v>
+        <v>1.6211090117473095</v>
       </c>
       <c r="D76" s="50">
         <f>IF($D$73&gt;0,MAX(1,$D$74/$D$73),1)</f>
-        <v>1.15310124070057</v>
+        <v>1.129366738319087</v>
       </c>
       <c r="E76" s="6" t="inlineStr">
         <is>
@@ -14111,11 +14115,11 @@
       </c>
       <c r="C78" s="21">
         <f>$C$77*$C$76</f>
-        <v>1623.7294734247916</v>
+        <v>1590.3079405241106</v>
       </c>
       <c r="D78" s="21">
         <f>$D$77*$D$76</f>
-        <v>1131.1923171272592</v>
+        <v>1107.9087702910244</v>
       </c>
       <c r="E78" s="6" t="inlineStr">
         <is>
@@ -14141,11 +14145,11 @@
       </c>
       <c r="C79" s="13">
         <f>IF(DATOS!$C$57="SÍ",0.9,1)*$C$21*DATOS!$C$60</f>
-        <v>2.62299652027786</v>
+        <v>2.56900688349684</v>
       </c>
       <c r="D79" s="13">
         <f>IF(DATOS!$C$57="SÍ",0.9,1)*$D$21*DATOS!$C$60</f>
-        <v>3.14450708339047</v>
+        <v>3.0797830953961505</v>
       </c>
       <c r="E79" s="6" t="inlineStr">
         <is>
@@ -14171,11 +14175,11 @@
       </c>
       <c r="C80" s="21">
         <f>IF($C$73&gt;0,MAX(1,$C$79/$C$73),1)</f>
-        <v>1.5083361243691</v>
+        <v>1.4772897547422885</v>
       </c>
       <c r="D80" s="21">
         <f>IF($D$73&gt;0,MAX(1,$D$79/$D$73),1)</f>
-        <v>1.15310124070057</v>
+        <v>1.129366738319087</v>
       </c>
       <c r="E80" s="6" t="inlineStr">
         <is>
@@ -14269,7 +14273,7 @@
       </c>
       <c r="C86" s="13">
         <f>DATOS!$C$60</f>
-        <v>17.49</v>
+        <v>17.13</v>
       </c>
       <c r="D86" s="53">
         <v>17.12906</v>
@@ -14281,7 +14285,7 @@
       </c>
       <c r="F86" s="44" t="inlineStr">
         <is>
-          <t>Tú: áreas tributarias (DATOS C60). Él: el peso que reporta STAAD (17,129 kg). Usa el W que imprime tu .anl para que el V mínimo y el V modal salgan de la misma masa.</t>
+          <t>Ya igualado: los dos usan el peso de STAAD (17.13 t). Esta diferencia ya no existe.</t>
         </is>
       </c>
       <c r="G86" s="48" t="inlineStr">
@@ -14416,7 +14420,7 @@
       </c>
       <c r="C91" s="13">
         <f>$C$74</f>
-        <v>2.878354285714286</v>
+        <v>2.8191085714285715</v>
       </c>
       <c r="D91" s="13">
         <f>D90*D86</f>
@@ -14475,7 +14479,7 @@
       </c>
       <c r="C93" s="21">
         <f>$C$76</f>
-        <v>1.6551778526246612</v>
+        <v>1.6211090117473095</v>
       </c>
       <c r="D93" s="21">
         <f>MAX(1,D91/D92)</f>
@@ -14517,7 +14521,7 @@
       </c>
       <c r="C95" s="13">
         <f>DATOS!$C$60</f>
-        <v>17.49</v>
+        <v>17.13</v>
       </c>
       <c r="D95" s="53">
         <v>17.12906</v>
@@ -14529,7 +14533,7 @@
       </c>
       <c r="F95" s="44" t="inlineStr">
         <is>
-          <t>Tú: áreas tributarias (DATOS C60). Él: el peso que reporta STAAD (17,129 kg). Usa el W que imprime tu .anl para que el V mínimo y el V modal salgan de la misma masa.</t>
+          <t>Ya igualado: los dos usan el peso de STAAD (17.13 t). Esta diferencia ya no existe.</t>
         </is>
       </c>
       <c r="G95" s="48" t="inlineStr">
@@ -14664,7 +14668,7 @@
       </c>
       <c r="C100" s="13">
         <f>$D$74</f>
-        <v>3.1445070833904656</v>
+        <v>3.0797830953961505</v>
       </c>
       <c r="D100" s="13">
         <f>D99*D95</f>
@@ -14723,7 +14727,7 @@
       </c>
       <c r="C102" s="21">
         <f>$D$76</f>
-        <v>1.153101240700574</v>
+        <v>1.129366738319087</v>
       </c>
       <c r="D102" s="21">
         <f>MAX(1,D100/D101)</f>
@@ -14785,11 +14789,11 @@
       </c>
       <c r="C104" s="13">
         <f>$C$78</f>
-        <v>1623.7294734247916</v>
+        <v>1590.3079405241106</v>
       </c>
       <c r="D104" s="13">
         <f>$D$78</f>
-        <v>1131.1923171272592</v>
+        <v>1107.9087702910244</v>
       </c>
       <c r="E104" s="6" t="inlineStr">
         <is>
@@ -14815,11 +14819,11 @@
       </c>
       <c r="C105" s="13">
         <f>STAAD!$C$18*$C$76</f>
-        <v>231.88214126345176</v>
+        <v>227.10926700073932</v>
       </c>
       <c r="D105" s="13">
         <f>STAAD!$D$18*$D$76</f>
-        <v>161.54371831594636</v>
+        <v>158.2186332048125</v>
       </c>
       <c r="E105" s="6" t="inlineStr">
         <is>
@@ -14845,11 +14849,11 @@
       </c>
       <c r="C106" s="55">
         <f>DATOS!$C$26/$C$12*$C$76</f>
-        <v>0.34049372968278724</v>
+        <v>0.33348528241658937</v>
       </c>
       <c r="D106" s="55">
         <f>DATOS!$C$26/$D$12*$D$76</f>
-        <v>0.23720939808697442</v>
+        <v>0.23232687188278361</v>
       </c>
       <c r="E106" s="6" t="inlineStr">
         <is>
@@ -22176,11 +22180,11 @@
       </c>
       <c r="C9" s="21">
         <f>COEFICIENTE!$C$24</f>
-        <v>2.91444057808651</v>
+        <v>2.8544520927742667</v>
       </c>
       <c r="D9" s="21">
         <f>COEFICIENTE!$D$24</f>
-        <v>3.49389675932274</v>
+        <v>3.421981217106834</v>
       </c>
       <c r="E9" s="6" t="s">
         <v>168</v>
@@ -22199,11 +22203,11 @@
       </c>
       <c r="C10" s="7">
         <f>COEFICIENTE!$C$24*9.80665</f>
-        <v>28.5808986950921</v>
+        <v>27.99261261560476</v>
       </c>
       <c r="D10" s="7">
         <f>COEFICIENTE!$D$24*9.80665</f>
-        <v>34.2634226548123</v>
+        <v>33.558172102740734</v>
       </c>
       <c r="E10" s="6" t="s">
         <v>339</v>
@@ -22222,7 +22226,7 @@
       </c>
       <c r="C11" s="13">
         <f>COEFICIENTE!$C$25*COEFICIENTE!$C$24</f>
-        <v>0.167900921703564</v>
+        <v>0.16444498506472552</v>
       </c>
       <c r="D11" s="13">
         <f>COEFICIENTE!$D$25*COEFICIENTE!$D$24</f>
@@ -22245,11 +22249,11 @@
       </c>
       <c r="C12" s="13">
         <f>COEFICIENTE!$C$27*DATOS!$C$60</f>
-        <v>2.87835428571429</v>
+        <v>2.8191085714285715</v>
       </c>
       <c r="D12" s="13">
         <f>COEFICIENTE!$D$27*DATOS!$C$60</f>
-        <v>3.14450708339047</v>
+        <v>3.0797830953961505</v>
       </c>
       <c r="E12" s="6" t="s">
         <v>168</v>
@@ -22291,11 +22295,11 @@
       </c>
       <c r="C14" s="13">
         <f>COEFICIENTE!$C$51</f>
-        <v>8.54045028571428</v>
+        <v>8.36466057142857</v>
       </c>
       <c r="D14" s="13">
         <f>COEFICIENTE!$D$51</f>
-        <v>8.54045028571428</v>
+        <v>8.36466057142857</v>
       </c>
       <c r="E14" s="6" t="s">
         <v>168</v>
@@ -22314,11 +22318,11 @@
       </c>
       <c r="C15" s="13">
         <f>COEFICIENTE!$C$54*DATOS!$C$61*IF(DATOS!$C$9="SÍ",COEFICIENTE!$C$64,1)</f>
-        <v>8.54045028571428</v>
+        <v>8.36466057142857</v>
       </c>
       <c r="D15" s="13">
         <f>COEFICIENTE!$D$54*DATOS!$C$61*IF(DATOS!$C$9="SÍ",COEFICIENTE!$D$64,1)</f>
-        <v>8.54045028571428</v>
+        <v>8.36466057142857</v>
       </c>
       <c r="E15" s="6" t="s">
         <v>168</v>
@@ -24998,11 +25002,11 @@
       </c>
       <c r="O15" s="21">
         <f>IF(STAAD!$C$17="ASCE 7-16",STAAD!$C$15,STAAD!$C$12)</f>
-        <v>2.87835428571429</v>
+        <v>2.8191085714285715</v>
       </c>
       <c r="P15" s="21">
         <f>IF(STAAD!$C$17="ASCE 7-16",STAAD!$D$15,STAAD!$D$12)</f>
-        <v>3.14450708339047</v>
+        <v>3.0797830953961505</v>
       </c>
       <c r="Q15" s="6" t="s">
         <v>168</v>
@@ -25187,7 +25191,7 @@
       </c>
       <c r="D19" s="30">
         <f t="shared" si="0"/>
-        <v>1210.69360162272</v>
+        <v>1210.6936016227182</v>
       </c>
       <c r="F19" s="24">
         <f>ESPECTROS!$B81</f>
@@ -26187,7 +26191,7 @@
       </c>
       <c r="D44" s="30">
         <f t="shared" si="3"/>
-        <v>1325.22019124599</v>
+        <v>1325.2201912459873</v>
       </c>
       <c r="F44" s="24">
         <f>ESPECTROS!$B106</f>
@@ -26225,7 +26229,7 @@
       </c>
       <c r="D45" s="30">
         <f t="shared" si="3"/>
-        <v>1299.10641140072</v>
+        <v>1299.1064114007158</v>
       </c>
       <c r="F45" s="24">
         <f>ESPECTROS!$B107</f>
@@ -26263,7 +26267,7 @@
       </c>
       <c r="D46" s="30">
         <f t="shared" si="3"/>
-        <v>1274.24217288049</v>
+        <v>1274.2421728804854</v>
       </c>
       <c r="F46" s="24">
         <f>ESPECTROS!$B108</f>
@@ -26301,7 +26305,7 @@
       </c>
       <c r="D47" s="30">
         <f t="shared" si="3"/>
-        <v>1250.53447889696</v>
+        <v>1250.5344788969583</v>
       </c>
       <c r="F47" s="24">
         <f>ESPECTROS!$B109</f>
@@ -26339,7 +26343,7 @@
       </c>
       <c r="D48" s="30">
         <f t="shared" si="3"/>
-        <v>1227.89959119257</v>
+        <v>1227.8995911925686</v>
       </c>
       <c r="F48" s="24">
         <f>ESPECTROS!$B110</f>
@@ -26415,7 +26419,7 @@
       </c>
       <c r="D50" s="30">
         <f t="shared" si="3"/>
-        <v>1179.50777925679</v>
+        <v>1179.507779256792</v>
       </c>
       <c r="F50" s="24">
         <f>ESPECTROS!$B112</f>
@@ -26529,7 +26533,7 @@
       </c>
       <c r="D53" s="30">
         <f t="shared" si="3"/>
-        <v>1128.40363685443</v>
+        <v>1128.4036368544316</v>
       </c>
       <c r="F53" s="24">
         <f>ESPECTROS!$B115</f>
@@ -26567,7 +26571,7 @@
       </c>
       <c r="D54" s="30">
         <f t="shared" si="3"/>
-        <v>1110.84048765984</v>
+        <v>1110.8404876598445</v>
       </c>
       <c r="F54" s="24">
         <f>ESPECTROS!$B116</f>
@@ -26605,7 +26609,7 @@
       </c>
       <c r="D55" s="30">
         <f t="shared" si="3"/>
-        <v>1093.94516506512</v>
+        <v>1093.9451650651185</v>
       </c>
       <c r="F55" s="24">
         <f>ESPECTROS!$B117</f>
@@ -26681,7 +26685,7 @@
       </c>
       <c r="D57" s="30">
         <f t="shared" si="3"/>
-        <v>1062.00228139343</v>
+        <v>1062.0022813934286</v>
       </c>
       <c r="F57" s="24">
         <f>ESPECTROS!$B119</f>
@@ -26719,7 +26723,7 @@
       </c>
       <c r="D58" s="30">
         <f t="shared" si="3"/>
-        <v>1046.88448980113</v>
+        <v>1046.8844898011257</v>
       </c>
       <c r="F58" s="24">
         <f>ESPECTROS!$B120</f>
@@ -26757,7 +26761,7 @@
       </c>
       <c r="D59" s="30">
         <f t="shared" si="3"/>
-        <v>1032.29346788803</v>
+        <v>1032.2934678880272</v>
       </c>
       <c r="F59" s="24">
         <f>ESPECTROS!$B121</f>
@@ -26795,7 +26799,7 @@
       </c>
       <c r="D60" s="30">
         <f t="shared" si="3"/>
-        <v>1018.20044881084</v>
+        <v>1018.2004488108361</v>
       </c>
       <c r="F60" s="24">
         <f>ESPECTROS!$B122</f>
@@ -26833,7 +26837,7 @@
       </c>
       <c r="D61" s="30">
         <f t="shared" si="3"/>
-        <v>1004.57878246495</v>
+        <v>1004.5787824649512</v>
       </c>
       <c r="F61" s="24">
         <f>ESPECTROS!$B123</f>

</xml_diff>